<commit_message>
Catalogo: de-para v2 com campos reais do describe + schema confirmado (precos custom ja existem, cadeia de dependencia)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/pricebooks-mulesoft/DePara_Catalogo_Mule.xlsx
+++ b/deploy/pricebooks-mulesoft/DePara_Catalogo_Mule.xlsx
@@ -115,7 +115,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">De-Para Catálogo GrupoQ -&gt; Salesforce (para MuleSoft)</t>
+          <t xml:space="preserve">De-Para Catalogo GrupoQ -&gt; Salesforce (para MuleSoft) - v2 (campos confirmados no describe)</t>
         </is>
       </c>
     </row>
@@ -125,7 +125,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objetivo: contrato de dados que o MuleSoft envia do SAP/QRM para popular o catálogo no Salesforce (sociedade C101 / Costa Rica). Catálogo STANDARD (sem EPC): specs de veículo em VehicleDefinition + campos custom; preço em Price Book.</t>
+          <t xml:space="preserve">Contrato de dados que o MuleSoft envia do SAP/QRM para popular o catalogo no Salesforce (sociedade C101 / Costa Rica). Catalogo STANDARD (sem EPC). API names confirmados via describe na org.</t>
         </is>
       </c>
     </row>
@@ -142,7 +142,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product2.ProductCode = código de material do SAP (MATNR). É a chave que o MuleSoft usa para UPSERT de tudo (produto, preço, inventário). Definir/confirmar como External Id em Product2 para upsert idempotente.</t>
+          <t xml:space="preserve">Product2.ProductCode = codigo de material do SAP (MATNR). Chave do UPSERT de tudo (produto, preco, inventario). Marcar ProductCode como External Id em Product2 para upsert idempotente. Para unidades fisicas, Vehicle.ExtlSystemVehicleIdentifier guarda a chave externa do SAP.</t>
         </is>
       </c>
     </row>
@@ -152,14 +152,14 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORDEM DE CARGA (dependências)</t>
+          <t xml:space="preserve">CADEIA DE DEPENDENCIA / ORDEM DE CARGA</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1) BusinessBrand (marca)  -&gt;  2) VehicleDefinition (ficha, por país)  -&gt;  3) Product2 (link marca/ficha, ProductCode=SAP)  -&gt;  4) PricebookEntry (preço no book C101)  -&gt;  5) Location (sucursales)  -&gt;  6) ProductItem / SerializedProduct (inventário)  -&gt;  7) Vehicle (unidades físicas / usados)</t>
+          <t xml:space="preserve">Product2 e a ANCORA. VehicleDefinition EXIGE ProductId (Product2). Vehicle EXIGE AssetId + VehicleDefinitionId + VIN. Ordem: 1) ProductCatalog/ProductCategory 2) BusinessBrand 3) Product2 (specs + ProductCode) 4) VehicleDefinition (ProductId + GeoCountryId) 5) PricebookEntry (book C101 + preco) 6) Location 7) ProductItem (estoque) 8) Asset (pre-req do Vehicle) 9) Vehicle (usados/unidades) 10) SerializedProduct.</t>
         </is>
       </c>
     </row>
@@ -169,14 +169,14 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FONTES</t>
+          <t xml:space="preserve">PRECO - CAMPOS CUSTOM JA EXISTEM (nao criar)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP = material master + inventário. QRM = variáveis de preço (lista, mínimo, exonerado, gastos, impostos, cashback). Derivado = calculado/fixo no mapeamento. Manual = definido pelo negócio.</t>
+          <t xml:space="preserve">O PricebookEntry ja tem os campos do QRM: PrecioExonerado__c, PrecioExoneradoMinimo__c, PrecioMinimoAsesor__c, Gastos__c, AplicaCashback__c, MontoCashback__c, VigenciaDesde__c. O de-para so mapeia o QRM para eles.</t>
         </is>
       </c>
     </row>
@@ -186,14 +186,31 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">A CONFIRMAR NO DESCRIBE (DESCRIBE-catalogo.apex)</t>
+          <t xml:space="preserve">FONTES</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Os campos marcados '(confirmar)' têm o API name a travar com o describe na org. Rodar o describe e ajustar a coluna 'Campo Salesforce'. Campos custom marcados 'CRIAR' ainda não existem e precisam ser criados.</t>
+          <t xml:space="preserve">SAP = material master + inventario. QRM = variaveis de preco (lista, minimo, exonerado, gastos, cashback). Derivado = calculado/fixo no mapeamento. Manual = negocio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OBSERVACOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EngineCubicCapacity (cilindrada) e STRING no VehicleDefinition. Specs marca/modelo/ano ficam no Product2 (MakeName/ModelName/ModelYear/ModelYearVersion/VehicleTrimLevel) e tambem no Vehicle. VehicleDefinition e enxuto (VehicleClass/ModelCode/EngineName/EngineCubicCapacity/GeoCountryId). Confirmar na agenda se novos entram como ProductItem/SerializedProduct (estoque) e usados como Vehicle+Asset (VIN individual).</t>
         </is>
       </c>
     </row>
@@ -205,12 +222,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="2" max="2" width="38" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="8" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
     <col min="8" max="8" width="40" customWidth="1"/>
   </cols>
   <sheetData>
@@ -269,7 +286,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BusinessBrand</t>
+          <t xml:space="preserve">ProductCatalog</t>
         </is>
       </c>
       <c r="B4" s="4"/>
@@ -283,7 +300,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">BusinessBrand</t>
+          <t xml:space="preserve">ProductCatalog</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -293,7 +310,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marca</t>
+          <t xml:space="preserve">Catalogo (linha)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -303,49 +320,49 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP/QRM</t>
+          <t xml:space="preserve">Manual/Derivado</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marca / Fabricante</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hyundai, Chevrolet, Isuzu...</t>
+          <t xml:space="preserve">Autos Novos, Motos, Repuestos, PA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">BusinessBrand</t>
+          <t xml:space="preserve">ProductCatalog</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ParentBrandId (confirmar)</t>
+          <t xml:space="preserve">Code</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marca pai</t>
+          <t xml:space="preserve">Codigo</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookup(BusinessBrand)</t>
+          <t xml:space="preserve">Text</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -358,16 +375,12 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Se houver hierarquia de marca</t>
-        </is>
-      </c>
+      <c r="H6" s="3"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinition</t>
+          <t xml:space="preserve">ProductCategory</t>
         </is>
       </c>
       <c r="B7" s="4"/>
@@ -381,7 +394,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinition</t>
+          <t xml:space="preserve">ProductCategory</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -391,7 +404,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ficha (marca modelo versão ano)</t>
+          <t xml:space="preserve">Categoria</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -401,411 +414,367 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">QRM/SAP</t>
+          <t xml:space="preserve">Manual/Derivado</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">concat</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ex.: Hyundai Tucson 2024 Limited</t>
+          <t xml:space="preserve">SUV/Sedan/Pickup; Filtros/Frenos</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinition</t>
+          <t xml:space="preserve">ProductCategory</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Make (confirmar)</t>
+          <t xml:space="preserve">CatalogId</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marca</t>
+          <t xml:space="preserve">Catalogo pai</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text/Lookup</t>
+          <t xml:space="preserve">Lookup(ProductCatalog)</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">confirmar</t>
+          <t xml:space="preserve">Sim (OBRIG)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">Derivado</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marca</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">confirmar se é texto ou lookup a BusinessBrand</t>
+          <t xml:space="preserve">match por Name/Code</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinition</t>
+          <t xml:space="preserve">ProductCategory</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Model (confirmar)</t>
+          <t xml:space="preserve">ParentCategoryId</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modelo</t>
+          <t xml:space="preserve">Categoria pai</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text</t>
+          <t xml:space="preserve">Lookup(ProductCategory)</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">confirmar</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">Derivado</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modelo</t>
-        </is>
-      </c>
-      <c r="H10" s="3"/>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hierarquia</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinition</t>
+          <t xml:space="preserve">ProductCategory</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Year / ModelYear (confirmar)</t>
+          <t xml:space="preserve">Code</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ano</t>
+          <t xml:space="preserve">Codigo</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Number</t>
+          <t xml:space="preserve">Text</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">confirmar</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">Derivado</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Año</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H11" s="3"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VehicleDefinition</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Trim / Version (confirmar)</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Versão</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SAP/QRM</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Versión</t>
-        </is>
-      </c>
-      <c r="H12" s="3"/>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BusinessBrand</t>
+        </is>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinition</t>
+          <t xml:space="preserve">BusinessBrand</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">BodyStyle/BodyType (confirmar)</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carroceria</t>
+          <t xml:space="preserve">Marca</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Picklist</t>
+          <t xml:space="preserve">Text</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">SAP/QRM</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tipo carroceria</t>
-        </is>
-      </c>
-      <c r="H13" s="3"/>
+          <t xml:space="preserve">Marca / Fabricante</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hyundai, Chevrolet, Isuzu...</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinition</t>
+          <t xml:space="preserve">BusinessBrand</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EngineCubicCapacity</t>
+          <t xml:space="preserve">ParentId</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cilindrada</t>
+          <t xml:space="preserve">Marca pai</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Number</t>
+          <t xml:space="preserve">Lookup(BusinessBrand)</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">Derivado</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cilindrada</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chave p/ Motos (evita custom)</t>
+          <t xml:space="preserve">hierarquia de marca</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VehicleDefinition</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FuelType / TransmissionType / DriveType (confirmar)</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Motorização/Transmissão/Tração</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Picklist</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SAP</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">specs</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">specs físicas</t>
-        </is>
-      </c>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product2</t>
+        </is>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinition</t>
+          <t xml:space="preserve">Product2</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GeoCountryId (confirmar)</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">País do catálogo</t>
+          <t xml:space="preserve">Nome comercial</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookup</t>
+          <t xml:space="preserve">Text</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí*</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivado</t>
+          <t xml:space="preserve">QRM/SAP</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">País (CR)</t>
+          <t xml:space="preserve">Descricao material</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">*chave do catálogo por país</t>
+          <t xml:space="preserve">marca modelo versao ano</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinition</t>
+          <t xml:space="preserve">Product2</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CurrencyIsoCode</t>
+          <t xml:space="preserve">ProductCode</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moeda</t>
+          <t xml:space="preserve">Codigo material (CHAVE)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Currency</t>
+          <t xml:space="preserve">Text</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Nao*</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivado</t>
+          <t xml:space="preserve">SAP</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">MATNR</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">por país (CRC/USD)</t>
+          <t xml:space="preserve">*CHAVE DE MATCH. External Id p/ upsert</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinition</t>
+          <t xml:space="preserve">Product2</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ProductId (confirmar link)</t>
+          <t xml:space="preserve">IsActive</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vínculo ao Product2</t>
+          <t xml:space="preserve">Ativo</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookup(Product2)</t>
+          <t xml:space="preserve">Checkbox</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">confirmar</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -820,23 +789,51 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">confirmar relação Definition&lt;-&gt;Product2 no describe</t>
+          <t xml:space="preserve">true</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Product2</t>
         </is>
       </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IsSerialized</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Serializa</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Checkbox</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Derivado</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">true p/ veiculos (habilita SerializedProduct)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -846,37 +843,37 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">BusinessBrandId</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nome comercial</t>
+          <t xml:space="preserve">Marca</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text</t>
+          <t xml:space="preserve">Lookup(BusinessBrand)</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">QRM/SAP</t>
+          <t xml:space="preserve">SAP/QRM</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Descrição material</t>
+          <t xml:space="preserve">Marca</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">marca modelo versão ano</t>
+          <t xml:space="preserve">match por Name da marca</t>
         </is>
       </c>
     </row>
@@ -888,22 +885,22 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ProductCode</t>
+          <t xml:space="preserve">MakeName</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Código material (CHAVE)</t>
+          <t xml:space="preserve">Marca (texto)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text</t>
+          <t xml:space="preserve">Text(80)</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -913,14 +910,10 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATNR</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">External Id p/ upsert. CHAVE DE MATCH de tudo</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Marca</t>
+        </is>
+      </c>
+      <c r="H21" s="3"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -930,39 +923,35 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">IsActive</t>
+          <t xml:space="preserve">ModelName</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ativo</t>
+          <t xml:space="preserve">Modelo</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checkbox</t>
+          <t xml:space="preserve">Text(80)</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivado</t>
+          <t xml:space="preserve">SAP</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Modelo</t>
+        </is>
+      </c>
+      <c r="H22" s="3"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -972,39 +961,35 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Family</t>
+          <t xml:space="preserve">ModelYear</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Linha</t>
+          <t xml:space="preserve">Ano</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Picklist</t>
+          <t xml:space="preserve">Number</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivado</t>
+          <t xml:space="preserve">SAP</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Autos/Motos/Repuestos/PA (sem EPC, usar Family)</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Ano</t>
+        </is>
+      </c>
+      <c r="H23" s="3"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1014,22 +999,22 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">BusinessBrandId</t>
+          <t xml:space="preserve">ModelYearVersion</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marca</t>
+          <t xml:space="preserve">Ano-versao</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookup(BusinessBrand)</t>
+          <t xml:space="preserve">Text(40)</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1039,14 +1024,10 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marca</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">match por Name da marca</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Version</t>
+        </is>
+      </c>
+      <c r="H24" s="3"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1056,39 +1037,35 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CurrencyIsoCode</t>
+          <t xml:space="preserve">VehicleTrimLevel</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moeda</t>
+          <t xml:space="preserve">Trim / versao</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Currency</t>
+          <t xml:space="preserve">Text(80)</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivado</t>
+          <t xml:space="preserve">SAP/QRM</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">por país</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Trim</t>
+        </is>
+      </c>
+      <c r="H25" s="3"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1098,12 +1075,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">StockKeepingUnit</t>
+          <t xml:space="preserve">ProductLineCode</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SKU</t>
+          <t xml:space="preserve">Codigo de linha</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1113,22 +1090,22 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">Derivado</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SKU</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">opcional</t>
+          <t xml:space="preserve">Autos/Motos/...</t>
         </is>
       </c>
     </row>
@@ -1140,32 +1117,32 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Description</t>
+          <t xml:space="preserve">ProductCategoryCode</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Descrição</t>
+          <t xml:space="preserve">Codigo categoria</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TextArea</t>
+          <t xml:space="preserve">Text</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP/QRM</t>
+          <t xml:space="preserve">Derivado</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Descrição</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H27" s="3"/>
@@ -1178,44 +1155,44 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">(custom) características (CRIAR se necessário)</t>
+          <t xml:space="preserve">CurrencyIsoCode</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Motorização/cor/tração de não-veículo</t>
+          <t xml:space="preserve">Moeda</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">varia</t>
+          <t xml:space="preserve">Currency</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">Derivado</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">specs</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">só se não couber no VehicleDefinition (peças)</t>
+          <t xml:space="preserve">por pais</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry</t>
+          <t xml:space="preserve">VehicleDefinition</t>
         </is>
       </c>
       <c r="B29" s="4"/>
@@ -1229,59 +1206,59 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry</t>
+          <t xml:space="preserve">VehicleDefinition</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pricebook2Id</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Book da sociedade</t>
+          <t xml:space="preserve">Ficha</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookup(Pricebook2)</t>
+          <t xml:space="preserve">Text</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivado</t>
+          <t xml:space="preserve">QRM/SAP</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">concat</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C101 (já criado). match por Name prefixo</t>
+          <t xml:space="preserve">Ex.: Hyundai Tucson 2024 Limited</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry</t>
+          <t xml:space="preserve">VehicleDefinition</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product2Id</t>
+          <t xml:space="preserve">ProductId</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Produto</t>
+          <t xml:space="preserve">Vinculo ao Product2</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1291,7 +1268,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Sim (OBRIG)</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -1306,234 +1283,222 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">match por ProductCode</t>
+          <t xml:space="preserve">EXIGIDO. match por ProductCode</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry</t>
+          <t xml:space="preserve">VehicleDefinition</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">UnitPrice</t>
+          <t xml:space="preserve">GeoCountryId</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preço de lista</t>
+          <t xml:space="preserve">Pais do catalogo</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Currency</t>
+          <t xml:space="preserve">Lookup(GeoCountry)</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">QRM</t>
+          <t xml:space="preserve">Derivado</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precio de lista</t>
+          <t xml:space="preserve">Pais (CR)</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">por moeda</t>
+          <t xml:space="preserve">chave do catalogo por pais</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry</t>
+          <t xml:space="preserve">VehicleDefinition</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CurrencyIsoCode</t>
+          <t xml:space="preserve">VehicleClass</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moeda</t>
+          <t xml:space="preserve">Classificacao</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Currency</t>
+          <t xml:space="preserve">Text</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">QRM</t>
+          <t xml:space="preserve">SAP</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moeda</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CRC / USD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Clase</t>
+        </is>
+      </c>
+      <c r="H33" s="3"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry</t>
+          <t xml:space="preserve">VehicleDefinition</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">IsActive</t>
+          <t xml:space="preserve">ModelCode</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ativo</t>
+          <t xml:space="preserve">Codigo modelo</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checkbox</t>
+          <t xml:space="preserve">Text</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivado</t>
+          <t xml:space="preserve">SAP</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Cod. modelo</t>
+        </is>
+      </c>
+      <c r="H34" s="3"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry</t>
+          <t xml:space="preserve">VehicleDefinition</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">UseStandardPrice</t>
+          <t xml:space="preserve">EngineName</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usa preço padrão</t>
+          <t xml:space="preserve">Motor</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checkbox</t>
+          <t xml:space="preserve">Text</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivado</t>
+          <t xml:space="preserve">SAP</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">false</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Motor</t>
+        </is>
+      </c>
+      <c r="H35" s="3"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry</t>
+          <t xml:space="preserve">VehicleDefinition</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PrecioMinimo__c (CRIAR)</t>
+          <t xml:space="preserve">EngineCubicCapacity</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preço mínimo</t>
+          <t xml:space="preserve">Cilindrada</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Currency</t>
+          <t xml:space="preserve">Text(255)</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">QRM</t>
+          <t xml:space="preserve">SAP</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precio mínimo</t>
+          <t xml:space="preserve">Cilindrada</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">campo custom a criar</t>
+          <t xml:space="preserve">e STRING; chave p/ Motos</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry</t>
+          <t xml:space="preserve">VehicleDefinition</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PrecioExonerado__c (CRIAR)</t>
+          <t xml:space="preserve">CurrencyIsoCode</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preço exonerado</t>
+          <t xml:space="preserve">Moeda</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1543,29 +1508,25 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">QRM</t>
+          <t xml:space="preserve">Derivado</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precio exonerado</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">campo custom a criar</t>
-        </is>
-      </c>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H37" s="3"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B38" s="4"/>
@@ -1579,32 +1540,32 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">Pricebook2Id</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Identificação</t>
+          <t xml:space="preserve">Book da sociedade</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text</t>
+          <t xml:space="preserve">Lookup(Pricebook2)</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Sim (OBRIG)</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">Derivado</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -1612,84 +1573,88 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="H39" s="3"/>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C101 (ja existe)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleIdentificationNumber</t>
+          <t xml:space="preserve">Product2Id</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VIN</t>
+          <t xml:space="preserve">Produto</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text</t>
+          <t xml:space="preserve">Lookup(Product2)</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No*</t>
+          <t xml:space="preserve">Sim (OBRIG)</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">Derivado</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VIN</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">*chave da unidade física</t>
+          <t xml:space="preserve">match por ProductCode</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleRegistrationNumber</t>
+          <t xml:space="preserve">UnitPrice</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Placa</t>
+          <t xml:space="preserve">Preco de lista</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text</t>
+          <t xml:space="preserve">Currency</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Sim (OBRIG)</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">QRM</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Placa</t>
+          <t xml:space="preserve">Precio de lista</t>
         </is>
       </c>
       <c r="H41" s="3"/>
@@ -1697,65 +1662,69 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ConditionType</t>
+          <t xml:space="preserve">CurrencyIsoCode</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condição</t>
+          <t xml:space="preserve">Moeda</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Picklist</t>
+          <t xml:space="preserve">Currency</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP/Derivado</t>
+          <t xml:space="preserve">QRM</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">New/Used</t>
-        </is>
-      </c>
-      <c r="H42" s="3"/>
+          <t xml:space="preserve">Moeda</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CRC / USD</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinitionId (confirmar)</t>
+          <t xml:space="preserve">UseStandardPrice</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ficha técnica</t>
+          <t xml:space="preserve">Usa preco padrao</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookup(VehicleDefinition)</t>
+          <t xml:space="preserve">Checkbox</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -1770,66 +1739,66 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">liga a unidade à ficha</t>
+          <t xml:space="preserve">false</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mileage (confirmar)</t>
+          <t xml:space="preserve">PrecioExonerado__c</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quilometragem</t>
+          <t xml:space="preserve">Preco exonerado</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Number</t>
+          <t xml:space="preserve">Currency</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">QRM</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Km</t>
+          <t xml:space="preserve">Precio exonerado</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">usados</t>
+          <t xml:space="preserve">JA EXISTE</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">AverageMarketValue / MarketPrice (confirmar)</t>
+          <t xml:space="preserve">PrecioExoneradoMinimo__c</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valor de mercado</t>
+          <t xml:space="preserve">Preco exonerado minimo</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1839,233 +1808,273 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">QRM/Avalúo</t>
+          <t xml:space="preserve">QRM</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Precio exon. minimo</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">usados</t>
+          <t xml:space="preserve">JA EXISTE</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Status (confirmar)</t>
+          <t xml:space="preserve">PrecioMinimoAsesor__c</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Estado</t>
+          <t xml:space="preserve">Preco minimo asesor</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Picklist</t>
+          <t xml:space="preserve">Currency</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">QRM</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Estado</t>
-        </is>
-      </c>
-      <c r="H46" s="3"/>
+          <t xml:space="preserve">Precio minimo</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JA EXISTE</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Location</t>
-        </is>
-      </c>
-      <c r="B47" s="4"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PricebookEntry</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gastos__c</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gastos</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Currency</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QRM</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gastos</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JA EXISTE</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Location</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">AplicaCashback__c</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sucursal / almacén</t>
+          <t xml:space="preserve">Aplica cashback</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text</t>
+          <t xml:space="preserve">Checkbox</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">QRM</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Centro/Almacén</t>
-        </is>
-      </c>
-      <c r="H48" s="3"/>
+          <t xml:space="preserve">Cashback?</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JA EXISTE</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ProductItem</t>
-        </is>
-      </c>
-      <c r="B49" s="4"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PricebookEntry</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MontoCashback__c</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monto cashback</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Currency</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QRM</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cashback</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JA EXISTE</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ProductItem</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product2Id</t>
+          <t xml:space="preserve">VigenciaDesde__c</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Produto</t>
+          <t xml:space="preserve">Vigencia desde</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookup(Product2)</t>
+          <t xml:space="preserve">Date</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivado</t>
+          <t xml:space="preserve">QRM</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Vigencia</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">match ProductCode</t>
+          <t xml:space="preserve">JA EXISTE</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ProductItem</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LocationId</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Local</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lookup(Location)</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sí</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SAP</t>
-        </is>
-      </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Centro</t>
-        </is>
-      </c>
-      <c r="H51" s="3"/>
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Location</t>
+        </is>
+      </c>
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+      <c r="G51" s="4"/>
+      <c r="H51" s="4"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ProductItem</t>
+          <t xml:space="preserve">Location</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">QuantityOnHand</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Estoque</t>
+          <t xml:space="preserve">Sucursal / almacen</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Number</t>
+          <t xml:space="preserve">Text</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
@@ -2075,146 +2084,1118 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stock</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">por local</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Centro/Almacen</t>
+        </is>
+      </c>
+      <c r="H52" s="3"/>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SerializedProduct</t>
-        </is>
-      </c>
-      <c r="B53" s="4"/>
-      <c r="C53" s="4"/>
-      <c r="D53" s="4"/>
-      <c r="E53" s="4"/>
-      <c r="F53" s="4"/>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Location</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LocationType</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tipo de local</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Picklist</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sim (OBRIG)</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Derivado</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ex.: Warehouse/Site</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SerializedProduct</t>
+          <t xml:space="preserve">Location</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SerialNumber</t>
+          <t xml:space="preserve">ParentLocationId</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Serie / VIN</t>
+          <t xml:space="preserve">Local pai</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text</t>
+          <t xml:space="preserve">Lookup(Location)</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí</t>
+          <t xml:space="preserve">Nao</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP</t>
+          <t xml:space="preserve">Derivado</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VIN/Serie</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">unidade serializada</t>
+          <t xml:space="preserve">hierarquia</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Location</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AccountId</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conta da sucursal</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lookup(Account)</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Derivado</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H55" s="3"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ProductItem</t>
+        </is>
+      </c>
+      <c r="B56" s="4"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="4"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4"/>
+      <c r="G56" s="4"/>
+      <c r="H56" s="4"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ProductItem</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LocationId</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lookup(Location)</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sim (OBRIG)</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Centro</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">match por Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ProductItem</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product2Id</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Produto</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lookup(Product2)</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sim (OBRIG)</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Derivado</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">match ProductCode</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ProductItem</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QuantityOnHand</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estoque</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sim (OBRIG)</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">por local</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ProductItem</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QuantityUnitOfMeasure</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UoM</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Picklist</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UoM</t>
+        </is>
+      </c>
+      <c r="H60" s="3"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ProductItem</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SerialNumber</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Serie / VIN</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text(80)</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIN/Serie</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">se serializado</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asset</t>
+        </is>
+      </c>
+      <c r="B62" s="4"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4"/>
+      <c r="H62" s="4"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asset</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ativo</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 por unidade fisica</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asset</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product2Id</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Produto</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lookup(Product2)</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Derivado</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">match ProductCode</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asset</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SerialNumber</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Serie / VIN</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIN</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">confirmar campos de Asset no describe</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehicle</t>
+        </is>
+      </c>
+      <c r="B66" s="4"/>
+      <c r="C66" s="4"/>
+      <c r="D66" s="4"/>
+      <c r="E66" s="4"/>
+      <c r="F66" s="4"/>
+      <c r="G66" s="4"/>
+      <c r="H66" s="4"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehicle</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identificacao</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H67" s="3"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehicle</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AssetId</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ativo</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lookup(Asset)</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sim (OBRIG)</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Derivado</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXIGIDO. criar Asset antes</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehicle</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VehicleDefinitionId</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ficha tecnica</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lookup(VehicleDefinition)</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sim (OBRIG)</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Derivado</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXIGIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehicle</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VehicleIdentificationNumber</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIN</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text(255)</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sim (OBRIG)</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIN</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXIGIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehicle</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VehicleRegistrationNumber</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Placa</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text(255)</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Placa</t>
+        </is>
+      </c>
+      <c r="H71" s="3"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehicle</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ConditionType</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condicao</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Picklist</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP/Derivado</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New/Used</t>
+        </is>
+      </c>
+      <c r="H72" s="3"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehicle</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MakeName / ModelName / ModelYear</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Specs</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marca/Modelo/Ano</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">denormalizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehicle</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MarketPrice / MarketPriceDate / MarketPriceSource</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor de mercado</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Currency/Date</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QRM/Avaluo</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">usados</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehicle</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">StockCode</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codigo de estoque</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock code</t>
+        </is>
+      </c>
+      <c r="H75" s="3"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehicle</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ExtlSystemVehicleIdentifier</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chave externa SAP</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text(255)</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID SAP</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chave externa da unidade</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehicle</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CurrentOwnerId</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dono atual</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lookup(Account)</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cliente</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">usados</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">SerializedProduct</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B78" s="4"/>
+      <c r="C78" s="4"/>
+      <c r="D78" s="4"/>
+      <c r="E78" s="4"/>
+      <c r="F78" s="4"/>
+      <c r="G78" s="4"/>
+      <c r="H78" s="4"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SerializedProduct</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Product2Id</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr">
+      <c r="C79" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Produto</t>
         </is>
       </c>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="D79" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Lookup(Product2)</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sí</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sim (OBRIG)</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Derivado</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G79" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="H55" s="3"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="H79" s="3"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">SerializedProduct</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Status (confirmar)</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estado</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Picklist</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SerialNumber</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Serie / VIN</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text(255)</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sim (OBRIG)</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">SAP</t>
         </is>
       </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estado</t>
-        </is>
-      </c>
-      <c r="H56" s="3"/>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIN/Serie</t>
+        </is>
+      </c>
+      <c r="H80" s="3"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SerializedProduct</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ProductItemId</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item de estoque</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lookup(ProductItem)</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Derivado</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H81" s="3"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SerializedProduct</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AssetId</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ativo</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lookup(Asset)</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Derivado</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H82" s="3"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>